<commit_message>
Documentation clean up and validation updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/CardiovascularValidation.xlsx
+++ b/data/human/adult/validation/Scenarios/CardiovascularValidation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\documentation\source\data\human\adult\validation\Scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\release_updates\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4329EC01-9852-4D92-9382-3B5BA343FEFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{936FE987-D5E0-4F9E-809E-055B755D5476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24510" yWindow="1110" windowWidth="32730" windowHeight="30885" tabRatio="695" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28170" yWindow="7365" windowWidth="24735" windowHeight="19980" tabRatio="695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="14" r:id="rId1"/>
@@ -1056,6 +1056,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1064,9 +1067,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1950,19 +1950,19 @@
         <v>54</v>
       </c>
       <c r="F16" s="27">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G16" s="21" t="s">
         <v>68</v>
       </c>
       <c r="H16" s="28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" s="21" t="s">
         <v>57</v>
       </c>
       <c r="J16" s="29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16" s="21" t="s">
         <v>58</v>
@@ -2334,21 +2334,21 @@
       </c>
       <c r="F27" s="27">
         <f>SUM(F3:F26)</f>
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="G27" s="21" t="s">
         <v>68</v>
       </c>
       <c r="H27" s="28">
         <f>SUM(H3:H26)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I27" s="21" t="s">
         <v>57</v>
       </c>
       <c r="J27" s="29">
         <f>SUM(J3:J26)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K27" s="21" t="s">
         <v>58</v>
@@ -2477,11 +2477,11 @@
       <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
       <c r="G1" t="s">
         <v>51</v>
       </c>
@@ -2639,11 +2639,11 @@
       <c r="C3" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="43" t="s">
         <v>99</v>
       </c>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
       <c r="G3" t="s">
         <v>51</v>
       </c>
@@ -2929,13 +2929,13 @@
       <c r="E1" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G1" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I1" s="38" t="s">
@@ -3209,13 +3209,13 @@
       <c r="E7" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="44" t="s">
+      <c r="F7" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G7" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="H7" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I7" s="38" t="s">
@@ -3489,13 +3489,13 @@
       <c r="E13" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="44" t="s">
+      <c r="F13" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G13" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="44" t="s">
+      <c r="H13" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I13" s="38" t="s">
@@ -3769,13 +3769,13 @@
       <c r="E19" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="44" t="s">
+      <c r="F19" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G19" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H19" s="44" t="s">
+      <c r="H19" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I19" s="38" t="s">
@@ -4049,13 +4049,13 @@
       <c r="E25" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="44" t="s">
+      <c r="F25" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G25" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H25" s="44" t="s">
+      <c r="H25" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I25" s="38" t="s">
@@ -4329,13 +4329,13 @@
       <c r="E31" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F31" s="44" t="s">
+      <c r="F31" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G31" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H31" s="44" t="s">
+      <c r="H31" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I31" s="38" t="s">
@@ -4609,13 +4609,13 @@
       <c r="E37" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F37" s="44" t="s">
+      <c r="F37" s="41" t="s">
         <v>91</v>
       </c>
       <c r="G37" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I37" s="38" t="s">
@@ -4889,13 +4889,13 @@
       <c r="E43" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F43" s="44" t="s">
+      <c r="F43" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G43" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H43" s="44" t="s">
+      <c r="H43" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I43" s="38" t="s">
@@ -5169,13 +5169,13 @@
       <c r="E50" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F50" s="44" t="s">
+      <c r="F50" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G50" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H50" s="44" t="s">
+      <c r="H50" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I50" s="38" t="s">
@@ -5449,13 +5449,13 @@
       <c r="E56" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F56" s="44" t="s">
+      <c r="F56" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G56" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H56" s="44" t="s">
+      <c r="H56" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I56" s="38" t="s">
@@ -5729,13 +5729,13 @@
       <c r="E62" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F62" s="44" t="s">
+      <c r="F62" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G62" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H62" s="44" t="s">
+      <c r="H62" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I62" s="38" t="s">
@@ -6009,13 +6009,13 @@
       <c r="E68" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F68" s="44" t="s">
+      <c r="F68" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G68" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H68" s="44" t="s">
+      <c r="H68" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I68" s="38" t="s">
@@ -6289,13 +6289,13 @@
       <c r="E74" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F74" s="44" t="s">
+      <c r="F74" s="41" t="s">
         <v>92</v>
       </c>
       <c r="G74" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="H74" s="44" t="s">
+      <c r="H74" s="41" t="s">
         <v>11</v>
       </c>
       <c r="I74" s="38" t="s">
@@ -7617,11 +7617,11 @@
       </c>
     </row>
     <row r="24" spans="2:24" ht="174" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="44" t="s">
         <v>193</v>
       </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
     </row>
     <row r="25" spans="2:24" x14ac:dyDescent="0.25">
       <c r="D25" s="20"/>
@@ -7812,11 +7812,11 @@
       <c r="C2" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
       <c r="G2" s="33" t="s">
         <v>51</v>
       </c>
@@ -7962,9 +7962,9 @@
       <c r="C4" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
       <c r="G4" s="33" t="s">
         <v>51</v>
       </c>
@@ -8033,9 +8033,9 @@
       <c r="C5" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
       <c r="G5" s="33" t="s">
         <v>51</v>
       </c>
@@ -8109,11 +8109,11 @@
       <c r="C8" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
       <c r="G8" s="33" t="s">
         <v>51</v>
       </c>
@@ -8259,9 +8259,9 @@
       <c r="C10" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="42"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
       <c r="G10" s="33" t="s">
         <v>51</v>
       </c>
@@ -8330,9 +8330,9 @@
       <c r="C11" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
       <c r="G11" s="33" t="s">
         <v>51</v>
       </c>
@@ -8406,11 +8406,11 @@
       <c r="C14" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
       <c r="G14" s="33" t="s">
         <v>51</v>
       </c>
@@ -8556,9 +8556,9 @@
       <c r="C16" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
       <c r="G16" s="33" t="s">
         <v>51</v>
       </c>
@@ -8627,9 +8627,9 @@
       <c r="C17" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
       <c r="G17" s="33" t="s">
         <v>51</v>
       </c>
@@ -8703,11 +8703,11 @@
       <c r="C21" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
       <c r="G21" s="33" t="s">
         <v>51</v>
       </c>
@@ -8853,9 +8853,9 @@
       <c r="C23" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="42"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
       <c r="G23" s="33" t="s">
         <v>51</v>
       </c>
@@ -8924,9 +8924,9 @@
       <c r="C24" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
       <c r="G24" s="33" t="s">
         <v>51</v>
       </c>
@@ -8995,9 +8995,9 @@
       <c r="C25" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="42"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="42"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
       <c r="G25" s="33" t="s">
         <v>51</v>
       </c>
@@ -9071,11 +9071,11 @@
       <c r="C29" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E29" s="41"/>
-      <c r="F29" s="41"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
       <c r="G29" s="33" t="s">
         <v>51</v>
       </c>
@@ -9221,9 +9221,9 @@
       <c r="C31" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="42"/>
-      <c r="E31" s="42"/>
-      <c r="F31" s="42"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="43"/>
+      <c r="F31" s="43"/>
       <c r="G31" s="33" t="s">
         <v>51</v>
       </c>
@@ -9292,9 +9292,9 @@
       <c r="C32" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="42"/>
+      <c r="D32" s="43"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
       <c r="G32" s="33" t="s">
         <v>51</v>
       </c>
@@ -9368,11 +9368,11 @@
       <c r="C36" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D36" s="41" t="s">
+      <c r="D36" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
       <c r="G36" s="33" t="s">
         <v>51</v>
       </c>
@@ -9518,9 +9518,9 @@
       <c r="C38" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D38" s="42"/>
-      <c r="E38" s="42"/>
-      <c r="F38" s="42"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
       <c r="G38" s="33" t="s">
         <v>51</v>
       </c>
@@ -9589,9 +9589,9 @@
       <c r="C39" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D39" s="42"/>
-      <c r="E39" s="42"/>
-      <c r="F39" s="42"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43"/>
       <c r="G39" s="33" t="s">
         <v>51</v>
       </c>
@@ -9665,11 +9665,11 @@
       <c r="C43" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D43" s="41" t="s">
+      <c r="D43" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
+      <c r="E43" s="42"/>
+      <c r="F43" s="42"/>
       <c r="G43" s="33" t="s">
         <v>51</v>
       </c>
@@ -9815,9 +9815,9 @@
       <c r="C45" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D45" s="42"/>
-      <c r="E45" s="42"/>
-      <c r="F45" s="42"/>
+      <c r="D45" s="43"/>
+      <c r="E45" s="43"/>
+      <c r="F45" s="43"/>
       <c r="G45" s="33" t="s">
         <v>51</v>
       </c>
@@ -9886,9 +9886,9 @@
       <c r="C46" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D46" s="42"/>
-      <c r="E46" s="42"/>
-      <c r="F46" s="42"/>
+      <c r="D46" s="43"/>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
       <c r="G46" s="33" t="s">
         <v>51</v>
       </c>
@@ -9957,9 +9957,9 @@
       <c r="C47" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D47" s="42"/>
-      <c r="E47" s="42"/>
-      <c r="F47" s="42"/>
+      <c r="D47" s="43"/>
+      <c r="E47" s="43"/>
+      <c r="F47" s="43"/>
       <c r="G47" s="33" t="s">
         <v>51</v>
       </c>
@@ -10033,11 +10033,11 @@
       <c r="C51" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D51" s="41" t="s">
+      <c r="D51" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E51" s="41"/>
-      <c r="F51" s="41"/>
+      <c r="E51" s="42"/>
+      <c r="F51" s="42"/>
       <c r="G51" s="33" t="s">
         <v>51</v>
       </c>
@@ -10183,9 +10183,9 @@
       <c r="C53" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D53" s="42"/>
-      <c r="E53" s="42"/>
-      <c r="F53" s="42"/>
+      <c r="D53" s="43"/>
+      <c r="E53" s="43"/>
+      <c r="F53" s="43"/>
       <c r="G53" s="33" t="s">
         <v>51</v>
       </c>
@@ -10254,9 +10254,9 @@
       <c r="C54" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
+      <c r="D54" s="43"/>
+      <c r="E54" s="43"/>
+      <c r="F54" s="43"/>
       <c r="G54" s="33" t="s">
         <v>51</v>
       </c>
@@ -10317,16 +10317,11 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D36:F36"/>
-    <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D10:F10"/>
     <mergeCell ref="D32:F32"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D14:F14"/>
@@ -10338,11 +10333,16 @@
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="D46:F46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10414,11 +10414,11 @@
       <c r="C2" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
       <c r="G2" s="33" t="s">
         <v>51</v>
       </c>
@@ -10576,11 +10576,11 @@
       <c r="C4" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="42" t="s">
+      <c r="D4" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
       <c r="G4" s="33" t="s">
         <v>51</v>
       </c>
@@ -10672,11 +10672,11 @@
       <c r="C7" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
       <c r="G7" s="33" t="s">
         <v>51</v>
       </c>
@@ -10834,11 +10834,11 @@
       <c r="C9" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="42" t="s">
+      <c r="D9" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
       <c r="G9" s="33" t="s">
         <v>51</v>
       </c>
@@ -10913,11 +10913,11 @@
       <c r="C10" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="42" t="s">
+      <c r="D10" s="43" t="s">
         <v>145</v>
       </c>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
       <c r="G10" s="33" t="s">
         <v>51</v>
       </c>

</xml_diff>